<commit_message>
feat(data): populate researched C7 Corvette Z51 used & wholesale OEM market quotes and proportional bundles
</commit_message>
<xml_diff>
--- a/Corvette-Z51-Repair-Comparison.xlsx
+++ b/Corvette-Z51-Repair-Comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="257">
   <si>
     <t>2015 CHEVROLET CORVETTE STINGRAY Z51 — REPAIR QUOTE &amp; USED PARTS COMPARISON</t>
   </si>
@@ -55,7 +55,7 @@
     <t xml:space="preserve">  ↳ Sourced Parts Only (Direct Comparison)</t>
   </si>
   <si>
-    <t>0 of 16 replaceable items currently sourced</t>
+    <t>14 of 16 replaceable items currently sourced</t>
   </si>
   <si>
     <t>Shop Labor Total (60.0 hrs + 6.625% Tax)</t>
@@ -106,102 +106,123 @@
     <t>84453011</t>
   </si>
   <si>
+    <t>eBay / Pacific Motors — Used OEM Coupe Right Quarter Panel</t>
+  </si>
+  <si>
+    <t>Watching / Quoted</t>
+  </si>
+  <si>
+    <t>C7 Stingray Coupe Right Rear Quarter Panel (SMC/Composite). If sourced in matching factory paint color, can potentially skip repaint (Lines 7 &amp; 8: 2.7u paint + 3.2h refinish).</t>
+  </si>
+  <si>
+    <t>Line #10: R Quarter Reinforcement</t>
+  </si>
+  <si>
+    <t>20980041</t>
+  </si>
+  <si>
+    <t>eBay / Corvette Salvage — Used OEM Reinforcement #20980041</t>
+  </si>
+  <si>
+    <t>Inner quarter panel reinforcement bracket</t>
+  </si>
+  <si>
+    <t>Line #11: R Drive Axle Differential Oil Cooler -M</t>
+  </si>
+  <si>
+    <t>22908627</t>
+  </si>
+  <si>
+    <t>eBay / C7 Salvage — Used OEM Z51 Differential Cooler #22908627</t>
+  </si>
+  <si>
+    <t>Z51 Package Differential Cooler mounted in rear quarter area</t>
+  </si>
+  <si>
+    <t>Line #16: R Upr Rear Susp Control Arm -M</t>
+  </si>
+  <si>
+    <t>84463637</t>
+  </si>
+  <si>
+    <t>[Bundle: Right Rear Suspension Knee Assembly (Lines 16–19)] eBay / Redline Auto Parts (Complete Right Rear Knee Assembly)</t>
+  </si>
+  <si>
+    <t>Great candidate for a Right Rear Suspension Knee Assembly bundle (with Lines 17, 18, 19)</t>
+  </si>
+  <si>
+    <t>Line #17: R Rear Susp Link -M</t>
+  </si>
+  <si>
+    <t>23175952</t>
+  </si>
+  <si>
+    <t>Right Rear Suspension Toe Link</t>
+  </si>
+  <si>
+    <t>Line #18: R Rear Susp Shock Absorber -M</t>
+  </si>
+  <si>
+    <t>84513886</t>
+  </si>
+  <si>
+    <t>Verify Z51 vs Magnetic Ride (FE3/FE4) RPO code on part #84513886 before ordering</t>
+  </si>
+  <si>
+    <t>Line #19: R Lwr Rear Susp Control Arm -M</t>
+  </si>
+  <si>
+    <t>20965286</t>
+  </si>
+  <si>
+    <t>High-value cast aluminum lower control arm ($887.11 OEM)</t>
+  </si>
+  <si>
+    <t>Line #20: Rear Susp Spring -M</t>
+  </si>
+  <si>
+    <t>22782496</t>
+  </si>
+  <si>
+    <t>eBay — Used C7 Rear Composite Transverse Leaf Spring #22782496</t>
+  </si>
+  <si>
+    <t>Transverse composite rear leaf spring (Z51 spec)</t>
+  </si>
+  <si>
+    <t>Line #23: R Rear Signal Lamp</t>
+  </si>
+  <si>
+    <t>23210930</t>
+  </si>
+  <si>
+    <t>eBay — Used OEM Right Rear Marker / Signal Lamp #23210930</t>
+  </si>
+  <si>
+    <t>Right rear side marker / signal lamp</t>
+  </si>
+  <si>
+    <t>Line #25: Rear Upr Bumper Cover</t>
+  </si>
+  <si>
+    <t>84411653</t>
+  </si>
+  <si>
+    <t>CorvetteSalvage.com / eBay — Used OEM Rear Upper Bumper Cover</t>
+  </si>
+  <si>
+    <t>Rear Upper Bumper Fascia. If sourced in matching factory paint color, toggle "Same Paint Color" to preview saving 4.0h Refinish + 3.3u Paint Materials.</t>
+  </si>
+  <si>
+    <t>Line #27: R Rear Combination Lamp Bezel</t>
+  </si>
+  <si>
+    <t>N.A.</t>
+  </si>
+  <si>
     <t>Shop Supplied (OEM New)</t>
   </si>
   <si>
-    <t>Need to Find</t>
-  </si>
-  <si>
-    <t>C7 Stingray Coupe Right Rear Quarter Panel (SMC/Composite). If sourced in matching factory paint color, can potentially skip repaint (Lines 7 &amp; 8: 2.7u paint + 3.2h refinish).</t>
-  </si>
-  <si>
-    <t>Line #10: R Quarter Reinforcement</t>
-  </si>
-  <si>
-    <t>20980041</t>
-  </si>
-  <si>
-    <t>Inner quarter panel reinforcement bracket</t>
-  </si>
-  <si>
-    <t>Line #11: R Drive Axle Differential Oil Cooler -M</t>
-  </si>
-  <si>
-    <t>22908627</t>
-  </si>
-  <si>
-    <t>Z51 Package Differential Cooler mounted in rear quarter area</t>
-  </si>
-  <si>
-    <t>Line #16: R Upr Rear Susp Control Arm -M</t>
-  </si>
-  <si>
-    <t>84463637</t>
-  </si>
-  <si>
-    <t>Great candidate for a Right Rear Suspension Knee Assembly bundle (with Lines 17, 18, 19)</t>
-  </si>
-  <si>
-    <t>Line #17: R Rear Susp Link -M</t>
-  </si>
-  <si>
-    <t>23175952</t>
-  </si>
-  <si>
-    <t>Right Rear Suspension Toe Link</t>
-  </si>
-  <si>
-    <t>Line #18: R Rear Susp Shock Absorber -M</t>
-  </si>
-  <si>
-    <t>84513886</t>
-  </si>
-  <si>
-    <t>Verify Z51 vs Magnetic Ride (FE3/FE4) RPO code on part #84513886 before ordering</t>
-  </si>
-  <si>
-    <t>Line #19: R Lwr Rear Susp Control Arm -M</t>
-  </si>
-  <si>
-    <t>20965286</t>
-  </si>
-  <si>
-    <t>High-value cast aluminum lower control arm ($887.11 OEM)</t>
-  </si>
-  <si>
-    <t>Line #20: Rear Susp Spring -M</t>
-  </si>
-  <si>
-    <t>22782496</t>
-  </si>
-  <si>
-    <t>Transverse composite rear leaf spring (Z51 spec)</t>
-  </si>
-  <si>
-    <t>Line #23: R Rear Signal Lamp</t>
-  </si>
-  <si>
-    <t>23210930</t>
-  </si>
-  <si>
-    <t>Right rear side marker / signal lamp</t>
-  </si>
-  <si>
-    <t>Line #25: Rear Upr Bumper Cover</t>
-  </si>
-  <si>
-    <t>84411653</t>
-  </si>
-  <si>
-    <t>Rear Upper Bumper Fascia. If sourced in matching factory paint color, toggle "Same Paint Color" to preview saving 4.0h Refinish + 3.3u Paint Materials.</t>
-  </si>
-  <si>
-    <t>Line #27: R Rear Combination Lamp Bezel</t>
-  </si>
-  <si>
-    <t>N.A.</t>
-  </si>
-  <si>
     <t>Shop / Existing</t>
   </si>
   <si>
@@ -214,6 +235,9 @@
     <t>84186343</t>
   </si>
   <si>
+    <t>eBay — Used OEM Rear Bumper Energy Absorber #84186343</t>
+  </si>
+  <si>
     <t>Rear bumper foam absorber</t>
   </si>
   <si>
@@ -223,6 +247,9 @@
     <t>84337474</t>
   </si>
   <si>
+    <t>eBay / Dino's Corvette Salvage — Used OEM Rear Impact Bar #84337474</t>
+  </si>
+  <si>
     <t>Aluminum rear crash bar / reinforcement beam</t>
   </si>
   <si>
@@ -232,6 +259,9 @@
     <t>285/30ZR20 (Z51)</t>
   </si>
   <si>
+    <t>[Bundle: Matching Rear Tire Pair — 285/30ZR20 Michelin ZP (Lines 36 &amp; 37)] United Tires (Utires.com) / eBay — Matching Used Pair (7.5/32"+ Tread)</t>
+  </si>
+  <si>
     <t>Z51 Rear Tire size: 285/30ZR20 Michelin Pilot Super Sport / Pilot Sport 4S ZP</t>
   </si>
   <si>
@@ -316,63 +346,117 @@
     <t>R Quarter Outer Panel</t>
   </si>
   <si>
+    <t>Standalone Used</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=C7+Corvette+Coupe+Right+Rear+Quarter+Panel+84453011+84054834</t>
+  </si>
+  <si>
+    <t>R Quarter Reinforcement</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=GM+20980041+Corvette</t>
+  </si>
+  <si>
+    <t>R Drive Axle Differential Oil Cooler -M</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=22908627+Corvette+Cooler</t>
+  </si>
+  <si>
+    <t>Rear Suspension</t>
+  </si>
+  <si>
+    <t>R Upr Rear Susp Control Arm -M</t>
+  </si>
+  <si>
+    <t>Bundle (14.04% share)</t>
+  </si>
+  <si>
+    <t>Right Rear Suspension Knee Assembly (Lines 16–19): eBay / Redline Auto Parts (Complete Right Rear Knee Assembly)</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=C7+Corvette+Right+Rear+Suspension+Knee+Assembly+20965286</t>
+  </si>
+  <si>
+    <t>R Rear Susp Link -M</t>
+  </si>
+  <si>
+    <t>Bundle (10.69% share)</t>
+  </si>
+  <si>
+    <t>R Rear Susp Shock Absorber -M</t>
+  </si>
+  <si>
+    <t>Bundle (14.5% share)</t>
+  </si>
+  <si>
+    <t>R Lwr Rear Susp Control Arm -M</t>
+  </si>
+  <si>
+    <t>Bundle (60.77% share)</t>
+  </si>
+  <si>
+    <t>Rear Susp Spring -M</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=22782496+Corvette+Rear+Leaf+Spring</t>
+  </si>
+  <si>
+    <t>Rear Lamps</t>
+  </si>
+  <si>
+    <t>R Rear Signal Lamp</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=23210930+Corvette</t>
+  </si>
+  <si>
+    <t>Rear Bumper</t>
+  </si>
+  <si>
+    <t>Rear Upr Bumper Cover</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=C7+Corvette+Rear+Upper+Bumper+Cover+84411653+23397592</t>
+  </si>
+  <si>
+    <t>R Rear Combination Lamp Bezel</t>
+  </si>
+  <si>
     <t>Shop OEM New</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>R Quarter Reinforcement</t>
-  </si>
-  <si>
-    <t>R Drive Axle Differential Oil Cooler -M</t>
-  </si>
-  <si>
-    <t>Rear Suspension</t>
-  </si>
-  <si>
-    <t>R Upr Rear Susp Control Arm -M</t>
-  </si>
-  <si>
-    <t>R Rear Susp Link -M</t>
-  </si>
-  <si>
-    <t>R Rear Susp Shock Absorber -M</t>
-  </si>
-  <si>
-    <t>R Lwr Rear Susp Control Arm -M</t>
-  </si>
-  <si>
-    <t>Rear Susp Spring -M</t>
-  </si>
-  <si>
-    <t>Rear Lamps</t>
-  </si>
-  <si>
-    <t>R Rear Signal Lamp</t>
-  </si>
-  <si>
-    <t>Rear Bumper</t>
-  </si>
-  <si>
-    <t>Rear Upr Bumper Cover</t>
-  </si>
-  <si>
-    <t>R Rear Combination Lamp Bezel</t>
-  </si>
-  <si>
     <t>Rear Bumper Energy Absorber</t>
   </si>
   <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=84186343+Corvette+Absorber</t>
+  </si>
+  <si>
     <t>Rear Bumper Impact Bar (Alum)</t>
   </si>
   <si>
+    <t>https://www.ebay.com/sch/i.html?_nkw=C7+Corvette+Rear+Impact+Bar+84337474+84180246+23136262</t>
+  </si>
+  <si>
     <t>Body Components (Tires)</t>
   </si>
   <si>
     <t>Right Rear Tire</t>
   </si>
   <si>
+    <t>Bundle (50% share)</t>
+  </si>
+  <si>
+    <t>Matching Rear Tire Pair — 285/30ZR20 Michelin ZP (Lines 36 &amp; 37): United Tires (Utires.com) / eBay — Matching Used Pair (7.5/32"+ Tread)</t>
+  </si>
+  <si>
+    <t>https://www.utires.com/tires/size/285-30r20/</t>
+  </si>
+  <si>
     <t>Left Rear Tire</t>
   </si>
   <si>
@@ -421,7 +505,10 @@
     <t>Part Savings vs OEM ($)</t>
   </si>
   <si>
-    <t>No bundles created yet. Create a bundle in the web app (e.g., Right Rear Suspension Knee Assembly) or enter rows here!</t>
+    <t>Right Rear Suspension Knee Assembly (Lines 16–19) (eBay / Redline Auto Parts (Complete Right Rear Knee Assembly))</t>
+  </si>
+  <si>
+    <t>Matching Rear Tire Pair — 285/30ZR20 Michelin ZP (Lines 36 &amp; 37) (United Tires (Utires.com) / eBay — Matching Used Pair (7.5/32"+ Tread))</t>
   </si>
   <si>
     <t>Code</t>
@@ -802,7 +889,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -832,6 +919,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1250,10 +1338,10 @@
         <v>12</v>
       </c>
       <c r="B7" s="8">
-        <v>0</v>
+        <v>7398.15</v>
       </c>
       <c r="C7" s="8">
-        <v>0</v>
+        <v>2922.59</v>
       </c>
       <c r="D7" s="8">
         <f>B7-C7</f>
@@ -1377,251 +1465,251 @@
         <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
         <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
         <v>31</v>
       </c>
       <c r="E17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
         <v>31</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
         <v>43</v>
-      </c>
-      <c r="C19" t="s">
-        <v>30</v>
       </c>
       <c r="D19" t="s">
         <v>31</v>
       </c>
       <c r="E19" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
         <v>31</v>
       </c>
       <c r="E20" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D21" t="s">
         <v>31</v>
       </c>
       <c r="E21" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="D22" t="s">
         <v>31</v>
       </c>
       <c r="E22" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D23" t="s">
         <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C24" t="s">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
         <v>31</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C25" t="s">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B26" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
       </c>
       <c r="E26" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D27" t="s">
         <v>31</v>
       </c>
       <c r="E27" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
         <v>31</v>
       </c>
       <c r="E28" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="C29" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
       </c>
       <c r="E29" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C30" t="s">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E30" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1659,7 +1747,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -1682,72 +1770,72 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B2" s="16">
         <v>0.06625</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="D4" s="17" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="S4" s="17" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1755,10 +1843,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D5" t="s">
         <v>29</v>
@@ -1773,14 +1861,20 @@
         <f>E5+F5</f>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I5" t="s">
-        <v>101</v>
-      </c>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="J5" s="6">
+        <v>350</v>
+      </c>
+      <c r="K5" s="6">
+        <v>125</v>
+      </c>
+      <c r="L5" s="6">
+        <v>31.47</v>
+      </c>
       <c r="M5" s="6">
         <f>IF(COUNT(J5:L5)&gt;0, SUM(J5:L5), "")</f>
       </c>
@@ -1794,10 +1888,10 @@
         <v>31</v>
       </c>
       <c r="Q5" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R5" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="S5" t="s">
         <v>32</v>
@@ -1808,10 +1902,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="D6" t="s">
         <v>34</v>
@@ -1826,14 +1920,20 @@
         <f>E6+F6</f>
       </c>
       <c r="H6" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I6" t="s">
-        <v>101</v>
-      </c>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
+        <v>35</v>
+      </c>
+      <c r="J6" s="6">
+        <v>38</v>
+      </c>
+      <c r="K6" s="6">
+        <v>12</v>
+      </c>
+      <c r="L6" s="6">
+        <v>3.31</v>
+      </c>
       <c r="M6" s="6">
         <f>IF(COUNT(J6:L6)&gt;0, SUM(J6:L6), "")</f>
       </c>
@@ -1847,13 +1947,13 @@
         <v>31</v>
       </c>
       <c r="Q6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R6" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="S6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -1861,13 +1961,13 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7" s="6">
         <v>581.12</v>
@@ -1879,14 +1979,20 @@
         <f>E7+F7</f>
       </c>
       <c r="H7" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I7" t="s">
-        <v>101</v>
-      </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
+        <v>39</v>
+      </c>
+      <c r="J7" s="6">
+        <v>175</v>
+      </c>
+      <c r="K7" s="6">
+        <v>20</v>
+      </c>
+      <c r="L7" s="6">
+        <v>12.92</v>
+      </c>
       <c r="M7" s="6">
         <f>IF(COUNT(J7:L7)&gt;0, SUM(J7:L7), "")</f>
       </c>
@@ -1900,13 +2006,13 @@
         <v>31</v>
       </c>
       <c r="Q7" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R7" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="S7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -1914,13 +2020,13 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E8" s="6">
         <v>204.93</v>
@@ -1932,14 +2038,20 @@
         <f>E8+F8</f>
       </c>
       <c r="H8" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="I8" t="s">
-        <v>101</v>
-      </c>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
+        <v>120</v>
+      </c>
+      <c r="J8" s="6">
+        <v>59.66</v>
+      </c>
+      <c r="K8" s="6">
+        <v>9.12</v>
+      </c>
+      <c r="L8" s="6">
+        <v>4.56</v>
+      </c>
       <c r="M8" s="6">
         <f>IF(COUNT(J8:L8)&gt;0, SUM(J8:L8), "")</f>
       </c>
@@ -1953,13 +2065,13 @@
         <v>31</v>
       </c>
       <c r="Q8" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R8" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="S8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -1967,13 +2079,13 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E9" s="6">
         <v>156.06</v>
@@ -1985,14 +2097,20 @@
         <f>E9+F9</f>
       </c>
       <c r="H9" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="I9" t="s">
-        <v>101</v>
-      </c>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
+        <v>120</v>
+      </c>
+      <c r="J9" s="6">
+        <v>45.43</v>
+      </c>
+      <c r="K9" s="6">
+        <v>6.95</v>
+      </c>
+      <c r="L9" s="6">
+        <v>3.47</v>
+      </c>
       <c r="M9" s="6">
         <f>IF(COUNT(J9:L9)&gt;0, SUM(J9:L9), "")</f>
       </c>
@@ -2006,13 +2124,13 @@
         <v>31</v>
       </c>
       <c r="Q9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R9" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="S9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2020,13 +2138,13 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E10" s="6">
         <v>211.73</v>
@@ -2038,14 +2156,20 @@
         <f>E10+F10</f>
       </c>
       <c r="H10" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="I10" t="s">
-        <v>101</v>
-      </c>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
+        <v>120</v>
+      </c>
+      <c r="J10" s="6">
+        <v>61.64</v>
+      </c>
+      <c r="K10" s="6">
+        <v>9.43</v>
+      </c>
+      <c r="L10" s="6">
+        <v>4.71</v>
+      </c>
       <c r="M10" s="6">
         <f>IF(COUNT(J10:L10)&gt;0, SUM(J10:L10), "")</f>
       </c>
@@ -2059,13 +2183,13 @@
         <v>31</v>
       </c>
       <c r="Q10" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R10" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="S10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -2073,13 +2197,13 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E11" s="6">
         <v>887.11</v>
@@ -2091,14 +2215,20 @@
         <f>E11+F11</f>
       </c>
       <c r="H11" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="I11" t="s">
-        <v>101</v>
-      </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
+        <v>120</v>
+      </c>
+      <c r="J11" s="6">
+        <v>258.26</v>
+      </c>
+      <c r="K11" s="6">
+        <v>39.5</v>
+      </c>
+      <c r="L11" s="6">
+        <v>19.73</v>
+      </c>
       <c r="M11" s="6">
         <f>IF(COUNT(J11:L11)&gt;0, SUM(J11:L11), "")</f>
       </c>
@@ -2112,13 +2242,13 @@
         <v>31</v>
       </c>
       <c r="Q11" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R11" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="S11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -2126,13 +2256,13 @@
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E12" s="6">
         <v>431.65</v>
@@ -2144,14 +2274,20 @@
         <f>E12+F12</f>
       </c>
       <c r="H12" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I12" t="s">
-        <v>101</v>
-      </c>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
+        <v>56</v>
+      </c>
+      <c r="J12" s="6">
+        <v>165</v>
+      </c>
+      <c r="K12" s="6">
+        <v>30</v>
+      </c>
+      <c r="L12" s="6">
+        <v>12.92</v>
+      </c>
       <c r="M12" s="6">
         <f>IF(COUNT(J12:L12)&gt;0, SUM(J12:L12), "")</f>
       </c>
@@ -2165,13 +2301,13 @@
         <v>31</v>
       </c>
       <c r="Q12" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R12" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="S12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -2179,13 +2315,13 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E13" s="6">
         <v>98.48</v>
@@ -2197,14 +2333,20 @@
         <f>E13+F13</f>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I13" t="s">
-        <v>101</v>
-      </c>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="J13" s="6">
+        <v>35</v>
+      </c>
+      <c r="K13" s="6">
+        <v>8</v>
+      </c>
+      <c r="L13" s="6">
+        <v>2.85</v>
+      </c>
       <c r="M13" s="6">
         <f>IF(COUNT(J13:L13)&gt;0, SUM(J13:L13), "")</f>
       </c>
@@ -2218,13 +2360,13 @@
         <v>31</v>
       </c>
       <c r="Q13" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R13" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
       <c r="S13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -2232,13 +2374,13 @@
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="D14" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E14" s="6">
         <v>1049.4</v>
@@ -2250,14 +2392,20 @@
         <f>E14+F14</f>
       </c>
       <c r="H14" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I14" t="s">
-        <v>101</v>
-      </c>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
+        <v>64</v>
+      </c>
+      <c r="J14" s="6">
+        <v>425</v>
+      </c>
+      <c r="K14" s="6">
+        <v>120</v>
+      </c>
+      <c r="L14" s="6">
+        <v>36.11</v>
+      </c>
       <c r="M14" s="6">
         <f>IF(COUNT(J14:L14)&gt;0, SUM(J14:L14), "")</f>
       </c>
@@ -2271,13 +2419,13 @@
         <v>31</v>
       </c>
       <c r="Q14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R14" t="s">
-        <v>101</v>
+        <v>135</v>
       </c>
       <c r="S14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -2285,13 +2433,13 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E15" s="6">
         <v>0</v>
@@ -2303,10 +2451,10 @@
         <f>E15+F15</f>
       </c>
       <c r="H15" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="I15" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
@@ -2321,16 +2469,16 @@
         <f>G15-N15</f>
       </c>
       <c r="P15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="Q15" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R15" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="S15" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -2338,13 +2486,13 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="D16" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E16" s="6">
         <v>273.01</v>
@@ -2356,14 +2504,20 @@
         <f>E16+F16</f>
       </c>
       <c r="H16" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I16" t="s">
-        <v>101</v>
-      </c>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
+        <v>73</v>
+      </c>
+      <c r="J16" s="6">
+        <v>85</v>
+      </c>
+      <c r="K16" s="6">
+        <v>18</v>
+      </c>
+      <c r="L16" s="6">
+        <v>6.82</v>
+      </c>
       <c r="M16" s="6">
         <f>IF(COUNT(J16:L16)&gt;0, SUM(J16:L16), "")</f>
       </c>
@@ -2377,13 +2531,13 @@
         <v>31</v>
       </c>
       <c r="Q16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R16" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
       <c r="S16" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -2391,13 +2545,13 @@
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="E17" s="6">
         <v>594.64</v>
@@ -2409,14 +2563,20 @@
         <f>E17+F17</f>
       </c>
       <c r="H17" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I17" t="s">
-        <v>101</v>
-      </c>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
+        <v>77</v>
+      </c>
+      <c r="J17" s="6">
+        <v>210</v>
+      </c>
+      <c r="K17" s="6">
+        <v>45</v>
+      </c>
+      <c r="L17" s="6">
+        <v>16.89</v>
+      </c>
       <c r="M17" s="6">
         <f>IF(COUNT(J17:L17)&gt;0, SUM(J17:L17), "")</f>
       </c>
@@ -2430,13 +2590,13 @@
         <v>31</v>
       </c>
       <c r="Q17" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R17" t="s">
-        <v>101</v>
+        <v>141</v>
       </c>
       <c r="S17" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -2444,13 +2604,13 @@
         <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="C18" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="D18" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="E18" s="6">
         <v>450</v>
@@ -2462,14 +2622,20 @@
         <f>E18+F18</f>
       </c>
       <c r="H18" t="s">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="I18" t="s">
-        <v>101</v>
-      </c>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
+        <v>145</v>
+      </c>
+      <c r="J18" s="6">
+        <v>195</v>
+      </c>
+      <c r="K18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
+        <v>12.92</v>
+      </c>
       <c r="M18" s="6">
         <f>IF(COUNT(J18:L18)&gt;0, SUM(J18:L18), "")</f>
       </c>
@@ -2483,13 +2649,13 @@
         <v>31</v>
       </c>
       <c r="Q18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R18" t="s">
-        <v>101</v>
+        <v>146</v>
       </c>
       <c r="S18" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -2497,13 +2663,13 @@
         <v>37</v>
       </c>
       <c r="B19" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="C19" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="E19" s="6">
         <v>450</v>
@@ -2515,14 +2681,20 @@
         <f>E19+F19</f>
       </c>
       <c r="H19" t="s">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="I19" t="s">
-        <v>101</v>
-      </c>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
+        <v>145</v>
+      </c>
+      <c r="J19" s="6">
+        <v>195</v>
+      </c>
+      <c r="K19" s="6">
+        <v>0</v>
+      </c>
+      <c r="L19" s="6">
+        <v>12.92</v>
+      </c>
       <c r="M19" s="6">
         <f>IF(COUNT(J19:L19)&gt;0, SUM(J19:L19), "")</f>
       </c>
@@ -2536,13 +2708,13 @@
         <v>31</v>
       </c>
       <c r="Q19" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R19" t="s">
-        <v>101</v>
+        <v>146</v>
       </c>
       <c r="S19" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -2550,13 +2722,13 @@
         <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="C20" t="s">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E20" s="6">
         <v>50</v>
@@ -2568,10 +2740,10 @@
         <f>E20+F20</f>
       </c>
       <c r="H20" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="I20" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
@@ -2586,30 +2758,30 @@
         <f>G20-N20</f>
       </c>
       <c r="P20" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="Q20" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R20" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="S20" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E21" s="19">
         <f>SUM(E5:E20)</f>
@@ -2621,10 +2793,10 @@
         <f>SUM(G5:G20)</f>
       </c>
       <c r="H21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J21" s="19">
         <f>SUM(J5:J20)</f>
@@ -2645,16 +2817,16 @@
         <f>SUM(O5:O20)</f>
       </c>
       <c r="P21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="Q21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="R21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="S21" s="18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2668,7 +2840,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2680,7 +2852,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2696,50 +2868,273 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" s="6">
+        <v>204.93</v>
+      </c>
+      <c r="E4" s="6">
+        <f>SUM($D$4:$D$7)</f>
+      </c>
+      <c r="F4" s="21">
+        <f>IF(E4&gt;0, D4/E4, 0)</f>
+      </c>
+      <c r="G4" s="6">
+        <v>522.46</v>
+      </c>
+      <c r="H4" s="6">
+        <f>ROUND(425*F4, 2)</f>
+      </c>
+      <c r="I4" s="6">
+        <f>ROUND(65*F4, 2)</f>
+      </c>
+      <c r="J4" s="6">
+        <f>ROUND(32.46*F4, 2)</f>
+      </c>
+      <c r="K4" s="6">
+        <f>ROUND(G4*F4, 2)</f>
+      </c>
+      <c r="L4" s="6">
+        <f>ROUND(D4*(1+0.06625), 2)-K4</f>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="6">
+        <v>156.06</v>
+      </c>
+      <c r="E5" s="6">
+        <f>SUM($D$4:$D$7)</f>
+      </c>
+      <c r="F5" s="21">
+        <f>IF(E5&gt;0, D5/E5, 0)</f>
+      </c>
+      <c r="G5" s="6">
+        <v>522.46</v>
+      </c>
+      <c r="H5" s="6">
+        <f>ROUND(425*F5, 2)</f>
+      </c>
+      <c r="I5" s="6">
+        <f>ROUND(65*F5, 2)</f>
+      </c>
+      <c r="J5" s="6">
+        <f>ROUND(32.46*F5, 2)</f>
+      </c>
+      <c r="K5" s="6">
+        <f>ROUND(G5*F5, 2)</f>
+      </c>
+      <c r="L5" s="6">
+        <f>ROUND(D5*(1+0.06625), 2)-K5</f>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
         <v>124</v>
       </c>
-      <c r="B3" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="D3" s="20" t="s">
+      <c r="D6" s="6">
+        <v>211.73</v>
+      </c>
+      <c r="E6" s="6">
+        <f>SUM($D$4:$D$7)</f>
+      </c>
+      <c r="F6" s="21">
+        <f>IF(E6&gt;0, D6/E6, 0)</f>
+      </c>
+      <c r="G6" s="6">
+        <v>522.46</v>
+      </c>
+      <c r="H6" s="6">
+        <f>ROUND(425*F6, 2)</f>
+      </c>
+      <c r="I6" s="6">
+        <f>ROUND(65*F6, 2)</f>
+      </c>
+      <c r="J6" s="6">
+        <f>ROUND(32.46*F6, 2)</f>
+      </c>
+      <c r="K6" s="6">
+        <f>ROUND(G6*F6, 2)</f>
+      </c>
+      <c r="L6" s="6">
+        <f>ROUND(D6*(1+0.06625), 2)-K6</f>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
         <v>126</v>
       </c>
-      <c r="E3" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>128</v>
-      </c>
-      <c r="G3" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>130</v>
-      </c>
-      <c r="I3" s="20" t="s">
-        <v>131</v>
-      </c>
-      <c r="J3" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>133</v>
-      </c>
-      <c r="L3" s="20" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>135</v>
+      <c r="D7" s="6">
+        <v>887.11</v>
+      </c>
+      <c r="E7" s="6">
+        <f>SUM($D$4:$D$7)</f>
+      </c>
+      <c r="F7" s="21">
+        <f>IF(E7&gt;0, D7/E7, 0)</f>
+      </c>
+      <c r="G7" s="6">
+        <v>522.46</v>
+      </c>
+      <c r="H7" s="6">
+        <f>ROUND(425*F7, 2)</f>
+      </c>
+      <c r="I7" s="6">
+        <f>ROUND(65*F7, 2)</f>
+      </c>
+      <c r="J7" s="6">
+        <f>ROUND(32.46*F7, 2)</f>
+      </c>
+      <c r="K7" s="6">
+        <f>ROUND(G7*F7, 2)</f>
+      </c>
+      <c r="L7" s="6">
+        <f>ROUND(D7*(1+0.06625), 2)-K7</f>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" s="6">
+        <v>450</v>
+      </c>
+      <c r="E9" s="6">
+        <f>SUM($D$9:$D$10)</f>
+      </c>
+      <c r="F9" s="21">
+        <f>IF(E9&gt;0, D9/E9, 0)</f>
+      </c>
+      <c r="G9" s="6">
+        <v>415.84</v>
+      </c>
+      <c r="H9" s="6">
+        <f>ROUND(390*F9, 2)</f>
+      </c>
+      <c r="I9" s="6">
+        <f>ROUND(0*F9, 2)</f>
+      </c>
+      <c r="J9" s="6">
+        <f>ROUND(25.84*F9, 2)</f>
+      </c>
+      <c r="K9" s="6">
+        <f>ROUND(G9*F9, 2)</f>
+      </c>
+      <c r="L9" s="6">
+        <f>ROUND(D9*(1+0.06625), 2)-K9</f>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>147</v>
+      </c>
+      <c r="D10" s="6">
+        <v>450</v>
+      </c>
+      <c r="E10" s="6">
+        <f>SUM($D$9:$D$10)</f>
+      </c>
+      <c r="F10" s="21">
+        <f>IF(E10&gt;0, D10/E10, 0)</f>
+      </c>
+      <c r="G10" s="6">
+        <v>415.84</v>
+      </c>
+      <c r="H10" s="6">
+        <f>ROUND(390*F10, 2)</f>
+      </c>
+      <c r="I10" s="6">
+        <f>ROUND(0*F10, 2)</f>
+      </c>
+      <c r="J10" s="6">
+        <f>ROUND(25.84*F10, 2)</f>
+      </c>
+      <c r="K10" s="6">
+        <f>ROUND(G10*F10, 2)</f>
+      </c>
+      <c r="L10" s="6">
+        <f>ROUND(D10*(1+0.06625), 2)-K10</f>
       </c>
     </row>
   </sheetData>
@@ -2770,44 +3165,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="C1" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="D1" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="F1" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="G1" s="21" t="s">
-        <v>141</v>
-      </c>
-      <c r="H1" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="I1" s="21" t="s">
+      <c r="A1" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="G1" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="H1" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="I1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="K1" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>145</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>97</v>
+      <c r="J1" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="K1" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="L1" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="M1" s="22" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2815,40 +3210,40 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>175</v>
       </c>
       <c r="C2" t="s">
-        <v>147</v>
+        <v>176</v>
       </c>
       <c r="D2" t="s">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="E2" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="F2" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G2">
         <v>4</v>
       </c>
       <c r="H2" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L2" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M2" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2856,40 +3251,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="C3" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D3" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="E3" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="F3" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G3">
         <v>0.9</v>
       </c>
       <c r="H3" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I3" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J3" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L3" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M3" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -2897,40 +3292,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D4" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="E4" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="F4" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L4" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2938,40 +3333,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D5" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
       <c r="E5" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="F5" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G5">
         <v>0.3</v>
       </c>
       <c r="H5" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I5" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J5" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L5" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M5" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -2979,40 +3374,40 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>194</v>
       </c>
       <c r="C6" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="D6" t="s">
-        <v>166</v>
+        <v>195</v>
       </c>
       <c r="E6" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="F6" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G6">
         <v>0.3</v>
       </c>
       <c r="H6" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L6" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3020,25 +3415,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>167</v>
+        <v>196</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F7" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G7">
         <v>2.5</v>
       </c>
       <c r="H7" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I7" t="s">
         <v>29</v>
@@ -3050,7 +3445,7 @@
         <v>1452.39</v>
       </c>
       <c r="L7" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M7" t="s">
         <v>32</v>
@@ -3061,40 +3456,40 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>172</v>
+        <v>201</v>
       </c>
       <c r="E8" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="F8" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G8">
         <v>2.2</v>
       </c>
       <c r="H8" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I8" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J8" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L8" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M8" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -3102,40 +3497,40 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>175</v>
+        <v>204</v>
       </c>
       <c r="E9" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="F9" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G9">
         <v>0.5</v>
       </c>
       <c r="H9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L9" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M9" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3143,40 +3538,40 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="E10" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="F10" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I10" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J10" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L10" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M10" t="s">
-        <v>177</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -3184,25 +3579,25 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>178</v>
+        <v>207</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="E11" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F11" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I11" t="s">
         <v>34</v>
@@ -3214,10 +3609,10 @@
         <v>97.96</v>
       </c>
       <c r="L11" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -3225,28 +3620,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>179</v>
+        <v>208</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="E12" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F12" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G12">
         <v>0.7</v>
       </c>
       <c r="H12" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -3255,10 +3650,10 @@
         <v>581.12</v>
       </c>
       <c r="L12" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -3266,40 +3661,40 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="C13" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="D13" t="s">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="E13" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="F13" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G13">
         <v>2</v>
       </c>
       <c r="H13" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I13" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J13" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L13" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M13" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -3307,40 +3702,40 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C14" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="D14" t="s">
-        <v>184</v>
+        <v>213</v>
       </c>
       <c r="E14" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="F14" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G14">
         <v>1.8</v>
       </c>
       <c r="H14" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L14" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -3348,40 +3743,40 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D15" t="s">
-        <v>185</v>
+        <v>214</v>
       </c>
       <c r="E15" t="s">
-        <v>186</v>
+        <v>215</v>
       </c>
       <c r="F15" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G15">
         <v>5</v>
       </c>
       <c r="H15" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I15" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J15" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L15" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M15" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -3389,40 +3784,40 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D16" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="F16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="G16">
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L16" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M16" t="s">
-        <v>189</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -3430,28 +3825,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D17" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="E17" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F17" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G17">
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -3460,10 +3855,10 @@
         <v>204.93</v>
       </c>
       <c r="L17" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M17" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -3471,28 +3866,28 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E18" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F18" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I18" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -3501,10 +3896,10 @@
         <v>156.06</v>
       </c>
       <c r="L18" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M18" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -3512,28 +3907,28 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>192</v>
+        <v>221</v>
       </c>
       <c r="C19" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="E19" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F19" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G19">
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I19" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -3542,10 +3937,10 @@
         <v>211.73</v>
       </c>
       <c r="L19" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M19" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -3553,28 +3948,28 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="E20" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F20" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G20">
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I20" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -3583,10 +3978,10 @@
         <v>887.11</v>
       </c>
       <c r="L20" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M20" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -3594,28 +3989,28 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>194</v>
+        <v>223</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D21" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F21" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G21">
         <v>4.8</v>
       </c>
       <c r="H21" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I21" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -3624,10 +4019,10 @@
         <v>431.65</v>
       </c>
       <c r="L21" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M21" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -3635,40 +4030,40 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="C22" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="E22" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="F22" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G22">
         <v>10</v>
       </c>
       <c r="H22" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I22" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J22" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L22" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M22" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -3676,40 +4071,40 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C23" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="D23" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="E23" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="F23" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G23">
         <v>2</v>
       </c>
       <c r="H23" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I23" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J23" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L23" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M23" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -3717,28 +4112,28 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="D24" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="E24" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F24" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G24">
         <v>0</v>
       </c>
       <c r="H24" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I24" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -3747,10 +4142,10 @@
         <v>98.48</v>
       </c>
       <c r="L24" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M24" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -3758,40 +4153,40 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C25" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D25" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="E25" t="s">
-        <v>186</v>
+        <v>215</v>
       </c>
       <c r="F25" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G25">
         <v>4.4</v>
       </c>
       <c r="H25" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="I25" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J25" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L25" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M25" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -3799,28 +4194,28 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="C26" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="E26" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F26" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G26">
         <v>0</v>
       </c>
       <c r="H26" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I26" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -3829,10 +4224,10 @@
         <v>1049.4</v>
       </c>
       <c r="L26" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M26" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
@@ -3840,40 +4235,40 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C27" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="E27" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="F27" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G27">
         <v>3.3</v>
       </c>
       <c r="H27" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I27" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J27" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L27" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M27" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -3881,40 +4276,40 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="C28" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D28" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="E28" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F28" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G28">
         <v>0</v>
       </c>
       <c r="H28" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I28" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="J28">
         <v>1</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L28" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M28" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
@@ -3922,28 +4317,28 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="C29" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D29" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="E29" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F29" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G29">
         <v>0.2</v>
       </c>
       <c r="H29" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I29" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="J29">
         <v>1</v>
@@ -3952,10 +4347,10 @@
         <v>273.01</v>
       </c>
       <c r="L29" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M29" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -3963,28 +4358,28 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
       <c r="C30" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D30" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="E30" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F30" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G30">
         <v>7.5</v>
       </c>
       <c r="H30" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I30" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="J30">
         <v>1</v>
@@ -3993,10 +4388,10 @@
         <v>594.64</v>
       </c>
       <c r="L30" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M30" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
@@ -4004,40 +4399,40 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C31" t="s">
-        <v>206</v>
+        <v>235</v>
       </c>
       <c r="D31" t="s">
-        <v>207</v>
+        <v>236</v>
       </c>
       <c r="E31" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="F31" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="G31">
         <v>0</v>
       </c>
       <c r="H31" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I31" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J31" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L31" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M31" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -4045,40 +4440,40 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C32" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="D32" t="s">
-        <v>211</v>
+        <v>240</v>
       </c>
       <c r="E32" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="F32" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G32">
         <v>2.3</v>
       </c>
       <c r="H32" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I32" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J32" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L32" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M32" t="s">
-        <v>213</v>
+        <v>242</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
@@ -4086,40 +4481,40 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>214</v>
+        <v>243</v>
       </c>
       <c r="C33" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="D33" t="s">
-        <v>215</v>
+        <v>244</v>
       </c>
       <c r="E33" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="F33" t="s">
-        <v>216</v>
+        <v>245</v>
       </c>
       <c r="G33">
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I33" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J33" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L33" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M33" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
@@ -4127,40 +4522,40 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>217</v>
+        <v>246</v>
       </c>
       <c r="C34" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="D34" t="s">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="E34" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="F34" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I34" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J34" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L34" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M34" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
@@ -4168,40 +4563,40 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>249</v>
       </c>
       <c r="C35" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="D35" t="s">
-        <v>221</v>
+        <v>250</v>
       </c>
       <c r="E35" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="F35" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I35" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J35" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L35" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M35" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
@@ -4209,40 +4604,40 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>222</v>
+        <v>251</v>
       </c>
       <c r="C36" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="D36" t="s">
-        <v>223</v>
+        <v>252</v>
       </c>
       <c r="E36" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="F36" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="G36">
         <v>0.3</v>
       </c>
       <c r="H36" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I36" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="J36" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L36" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="M36" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
@@ -4250,28 +4645,28 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="C37" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="D37" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="E37" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F37" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I37" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="J37">
         <v>1</v>
@@ -4280,10 +4675,10 @@
         <v>450</v>
       </c>
       <c r="L37" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M37" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
@@ -4291,28 +4686,28 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>226</v>
+        <v>255</v>
       </c>
       <c r="C38" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="D38" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="E38" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F38" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G38">
         <v>0</v>
       </c>
       <c r="H38" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I38" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="J38">
         <v>1</v>
@@ -4321,10 +4716,10 @@
         <v>450</v>
       </c>
       <c r="L38" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M38" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
@@ -4332,28 +4727,28 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>227</v>
+        <v>256</v>
       </c>
       <c r="C39" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="E39" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="F39" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G39">
         <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="I39" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -4362,10 +4757,10 @@
         <v>50</v>
       </c>
       <c r="L39" t="s">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="M39" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>